<commit_message>
Fix bug xe cơ động
</commit_message>
<xml_diff>
--- a/EPORTAL/App_Data/BM_09.QT20 Dondangkyxecodongnhathau.xlsx
+++ b/EPORTAL/App_Data/BM_09.QT20 Dondangkyxecodongnhathau.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\test\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SOFTWARE\EPORTAL\EPORTAL\App_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FDD657B-0296-4063-BE25-6DDA06F28AD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79CDA911-1496-4242-8A59-523978E33EC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="2520" windowWidth="24240" windowHeight="13020" xr2:uid="{46B31B07-A51E-47E9-9D50-BD8EC39AFAC0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{46B31B07-A51E-47E9-9D50-BD8EC39AFAC0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -385,7 +385,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -455,15 +455,28 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="5" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -927,7 +940,7 @@
     <col min="6" max="6" width="10.28515625" customWidth="1"/>
     <col min="7" max="7" width="9.42578125" customWidth="1"/>
     <col min="8" max="8" width="10.5703125" customWidth="1"/>
-    <col min="9" max="9" width="28.85546875" customWidth="1"/>
+    <col min="9" max="9" width="28.85546875" style="32" customWidth="1"/>
     <col min="10" max="10" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1004,14 +1017,14 @@
       </c>
       <c r="G5" s="23"/>
       <c r="H5" s="23"/>
-      <c r="I5" s="25" t="s">
+      <c r="I5" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="J5" s="27" t="s">
+      <c r="J5" s="25" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="33" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A6" s="22"/>
       <c r="B6" s="4" t="s">
         <v>9</v>
@@ -1032,8 +1045,8 @@
       <c r="H6" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="I6" s="26"/>
-      <c r="J6" s="27"/>
+      <c r="I6" s="27"/>
+      <c r="J6" s="25"/>
     </row>
     <row r="7" spans="1:10" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A7" s="7">
@@ -1046,7 +1059,7 @@
       <c r="F7" s="10"/>
       <c r="G7" s="9"/>
       <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
+      <c r="I7" s="28"/>
       <c r="J7" s="10"/>
     </row>
     <row r="8" spans="1:10" ht="16.5" x14ac:dyDescent="0.25">
@@ -1060,7 +1073,7 @@
       <c r="F8" s="10"/>
       <c r="G8" s="9"/>
       <c r="H8" s="9"/>
-      <c r="I8" s="9"/>
+      <c r="I8" s="28"/>
       <c r="J8" s="10"/>
     </row>
     <row r="9" spans="1:10" ht="16.5" x14ac:dyDescent="0.25">
@@ -1074,7 +1087,7 @@
       <c r="F9" s="9"/>
       <c r="G9" s="10"/>
       <c r="H9" s="9"/>
-      <c r="I9" s="9"/>
+      <c r="I9" s="28"/>
       <c r="J9" s="10"/>
     </row>
     <row r="10" spans="1:10" ht="16.5" x14ac:dyDescent="0.25">
@@ -1088,7 +1101,7 @@
       <c r="F10" s="10"/>
       <c r="G10" s="10"/>
       <c r="H10" s="10"/>
-      <c r="I10" s="10"/>
+      <c r="I10" s="29"/>
       <c r="J10" s="10"/>
     </row>
     <row r="11" spans="1:10" ht="16.5" x14ac:dyDescent="0.25">
@@ -1102,7 +1115,7 @@
       <c r="F11" s="10"/>
       <c r="G11" s="10"/>
       <c r="H11" s="10"/>
-      <c r="I11" s="10"/>
+      <c r="I11" s="29"/>
       <c r="J11" s="10"/>
     </row>
     <row r="12" spans="1:10" ht="16.5" x14ac:dyDescent="0.25">
@@ -1130,7 +1143,7 @@
       <c r="H13" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="I13" s="12"/>
+      <c r="I13" s="30"/>
       <c r="J13" s="12"/>
     </row>
     <row r="14" spans="1:10" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1146,7 +1159,7 @@
       </c>
       <c r="G14" s="13"/>
       <c r="H14" s="11"/>
-      <c r="I14" s="3" t="s">
+      <c r="I14" s="31" t="s">
         <v>19</v>
       </c>
       <c r="J14" s="13"/>

</xml_diff>